<commit_message>
Actualizacion automatica SIPREM y Casuistica GUAJIRA
</commit_message>
<xml_diff>
--- a/siprem_latest.xlsx
+++ b/siprem_latest.xlsx
@@ -29,7 +29,7 @@
     <t>FECHA</t>
   </si>
   <si>
-    <t>27/07/2026 a las 16:13:42</t>
+    <t>27/07/2026 a las 16:16:42</t>
   </si>
   <si>
     <t>Num_Lote</t>
@@ -63912,7 +63912,7 @@
         <v>0</v>
       </c>
       <c r="X693" s="4" t="s">
-        <v>267</v>
+        <v>1258</v>
       </c>
       <c r="Y693" s="4"/>
       <c r="Z693" s="4" t="s">

</xml_diff>